<commit_message>
Daily NSE scan: 2026-08-27
</commit_message>
<xml_diff>
--- a/output/2026-08-27/enriched_analysis.xlsx
+++ b/output/2026-08-27/enriched_analysis.xlsx
@@ -616,7 +616,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Gandhar Oil Refinery (India) Limited</t>
+          <t>GANDHAR OIL REFINERY (INDIA) LIMITED</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -663,13 +663,13 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>0.08</v>
+        <v>0.079</v>
       </c>
       <c r="Q2" t="n">
-        <v>2496</v>
+        <v>2512</v>
       </c>
       <c r="R2" t="n">
-        <v>8.58</v>
+        <v>8.65</v>
       </c>
       <c r="S2" t="n">
         <v>36</v>
@@ -740,19 +740,19 @@
         <v>95.20999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>55.67</v>
+        <v>55.78</v>
       </c>
       <c r="K3" t="n">
-        <v>71</v>
+        <v>70.7</v>
       </c>
       <c r="L3" t="n">
         <v>67.45999999999999</v>
       </c>
       <c r="M3" t="n">
-        <v>6.76</v>
+        <v>6.19</v>
       </c>
       <c r="N3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -760,13 +760,13 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>0.678</v>
+        <v>0.628</v>
       </c>
       <c r="Q3" t="n">
-        <v>997</v>
+        <v>985</v>
       </c>
       <c r="R3" t="n">
-        <v>28.5</v>
+        <v>28.2</v>
       </c>
       <c r="S3" t="n">
         <v>19</v>
@@ -860,10 +860,10 @@
         <v>0.039</v>
       </c>
       <c r="Q4" t="n">
-        <v>17118</v>
+        <v>17058</v>
       </c>
       <c r="R4" t="n">
-        <v>43.6</v>
+        <v>43.5</v>
       </c>
       <c r="S4" t="n">
         <v>83</v>
@@ -954,13 +954,13 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>0.024</v>
+        <v>0.022</v>
       </c>
       <c r="Q5" t="n">
-        <v>1870</v>
+        <v>1977</v>
       </c>
       <c r="R5" t="n">
-        <v>48.1</v>
+        <v>50.8</v>
       </c>
       <c r="S5" t="n">
         <v>35</v>
@@ -1051,13 +1051,13 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>0.093</v>
+        <v>0.095</v>
       </c>
       <c r="Q6" t="n">
-        <v>16215</v>
+        <v>15981</v>
       </c>
       <c r="R6" t="n">
-        <v>20.6</v>
+        <v>20.2</v>
       </c>
       <c r="S6" t="n">
         <v>16</v>
@@ -1148,13 +1148,13 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>0.333</v>
+        <v>0.33</v>
       </c>
       <c r="Q7" t="n">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="R7" t="n">
-        <v>8.91</v>
+        <v>9.02</v>
       </c>
       <c r="S7" t="n">
         <v>17</v>
@@ -1245,13 +1245,13 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>0.083</v>
+        <v>0.079</v>
       </c>
       <c r="Q8" t="n">
-        <v>988</v>
+        <v>1042</v>
       </c>
       <c r="R8" t="n">
-        <v>13.3</v>
+        <v>14</v>
       </c>
       <c r="S8" t="n">
         <v>55</v>
@@ -1345,10 +1345,10 @@
         <v>0.007</v>
       </c>
       <c r="Q9" t="n">
-        <v>5933</v>
+        <v>5856</v>
       </c>
       <c r="R9" t="n">
-        <v>10</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="S9" t="n">
         <v>43</v>
@@ -1387,111 +1387,113 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>CHEMBONDCH</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PNGS Reva Diamond Jewellery Limited</t>
+          <t>CHEMBOND CHEMICALS LIMITED</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Buy on Breakout</t>
+          <t>Strong Buy Setup</t>
         </is>
       </c>
       <c r="E10" t="n">
         <v>20</v>
       </c>
       <c r="F10" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="G10" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>542.9</v>
+        <v>269.84</v>
       </c>
       <c r="J10" t="n">
-        <v>390.61</v>
+        <v>243.52</v>
       </c>
       <c r="K10" t="n">
-        <v>39</v>
+        <v>10.8</v>
       </c>
       <c r="L10" t="n">
-        <v>63.09</v>
+        <v>67.65000000000001</v>
       </c>
       <c r="M10" t="n">
-        <v>8.02</v>
+        <v>1.11</v>
       </c>
       <c r="N10" t="n">
         <v>3</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>25-08-2026</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>0.467</v>
+        <v>0.155</v>
       </c>
       <c r="Q10" t="n">
-        <v>1718</v>
+        <v>715</v>
       </c>
       <c r="R10" t="n">
-        <v>20.4</v>
+        <v>59.8</v>
       </c>
       <c r="S10" t="n">
-        <v>581</v>
+        <v>3</v>
       </c>
       <c r="T10" t="n">
-        <v>34</v>
+        <v>2.99</v>
       </c>
       <c r="U10" t="n">
-        <v>881</v>
+        <v>97</v>
       </c>
       <c r="V10" t="n">
-        <v>8.58</v>
+        <v>1</v>
       </c>
       <c r="W10" t="n">
-        <v>22</v>
+        <v>11.6</v>
       </c>
       <c r="X10" t="n">
-        <v>0.33</v>
+        <v>0</v>
       </c>
       <c r="Y10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z10" t="n">
-        <v>29</v>
+        <v>16.21</v>
       </c>
       <c r="AA10" t="n">
-        <v>460.42</v>
-      </c>
-      <c r="AB10" t="inlineStr"/>
+        <v>244.22</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>177.4</v>
+      </c>
       <c r="AC10" t="n">
-        <v>31.9</v>
+        <v>74.2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CHEMBONDCH</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CHEMBOND CHEMICALS LIMITED</t>
+          <t>PNGS Reva Diamond Jewellery Limited</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1502,78 +1504,76 @@
         <v>20</v>
       </c>
       <c r="F11" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="G11" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H11" t="n">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>269.84</v>
+        <v>542.9</v>
       </c>
       <c r="J11" t="n">
-        <v>243.52</v>
+        <v>390.61</v>
       </c>
       <c r="K11" t="n">
-        <v>10.8</v>
+        <v>39</v>
       </c>
       <c r="L11" t="n">
-        <v>67.65000000000001</v>
+        <v>63.09</v>
       </c>
       <c r="M11" t="n">
-        <v>1.11</v>
+        <v>8.02</v>
       </c>
       <c r="N11" t="n">
         <v>3</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>25-08-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>0.152</v>
+        <v>0.464</v>
       </c>
       <c r="Q11" t="n">
-        <v>730</v>
+        <v>1727</v>
       </c>
       <c r="R11" t="n">
-        <v>61</v>
+        <v>20.5</v>
       </c>
       <c r="S11" t="n">
-        <v>3</v>
+        <v>581</v>
       </c>
       <c r="T11" t="n">
-        <v>2.99</v>
+        <v>34</v>
       </c>
       <c r="U11" t="n">
-        <v>97</v>
+        <v>881</v>
       </c>
       <c r="V11" t="n">
-        <v>1</v>
+        <v>8.58</v>
       </c>
       <c r="W11" t="n">
-        <v>11.6</v>
+        <v>22</v>
       </c>
       <c r="X11" t="n">
-        <v>0</v>
+        <v>0.33</v>
       </c>
       <c r="Y11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z11" t="n">
-        <v>16.21</v>
+        <v>29</v>
       </c>
       <c r="AA11" t="n">
-        <v>244.22</v>
-      </c>
-      <c r="AB11" t="n">
-        <v>177.4</v>
-      </c>
+        <v>460.42</v>
+      </c>
+      <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="n">
-        <v>74.2</v>
+        <v>31.9</v>
       </c>
     </row>
     <row r="12">
@@ -1634,7 +1634,7 @@
         <v>0.006</v>
       </c>
       <c r="Q12" t="n">
-        <v>4094</v>
+        <v>4070</v>
       </c>
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="n">
@@ -1726,13 +1726,13 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>0.08</v>
+        <v>0.077</v>
       </c>
       <c r="Q13" t="n">
-        <v>427</v>
+        <v>444</v>
       </c>
       <c r="R13" t="n">
-        <v>12.6</v>
+        <v>13.1</v>
       </c>
       <c r="S13" t="n">
         <v>-8</v>
@@ -1823,13 +1823,13 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>0.476</v>
+        <v>0.475</v>
       </c>
       <c r="Q14" t="n">
-        <v>1149</v>
+        <v>1151</v>
       </c>
       <c r="R14" t="n">
-        <v>58.5</v>
+        <v>58.6</v>
       </c>
       <c r="S14" t="n">
         <v>21</v>
@@ -2017,13 +2017,13 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>0.128</v>
+        <v>0.133</v>
       </c>
       <c r="Q16" t="n">
-        <v>390</v>
+        <v>375</v>
       </c>
       <c r="R16" t="n">
-        <v>6.29</v>
+        <v>6.04</v>
       </c>
       <c r="S16" t="n">
         <v>118</v>
@@ -2110,13 +2110,13 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>0.361</v>
+        <v>0.354</v>
       </c>
       <c r="Q17" t="n">
-        <v>410</v>
+        <v>418</v>
       </c>
       <c r="R17" t="n">
-        <v>38.1</v>
+        <v>38.7</v>
       </c>
       <c r="S17" t="n">
         <v>21</v>
@@ -2207,13 +2207,13 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>0.237</v>
+        <v>0.241</v>
       </c>
       <c r="Q18" t="n">
-        <v>2640</v>
+        <v>2588</v>
       </c>
       <c r="R18" t="n">
-        <v>21.6</v>
+        <v>21.2</v>
       </c>
       <c r="S18" t="n">
         <v>8</v>
@@ -2304,13 +2304,13 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>0.209</v>
+        <v>0.205</v>
       </c>
       <c r="Q19" t="n">
-        <v>1443</v>
+        <v>1470</v>
       </c>
       <c r="R19" t="n">
-        <v>50.3</v>
+        <v>51.2</v>
       </c>
       <c r="S19" t="n">
         <v>7</v>
@@ -2401,13 +2401,13 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>0.465</v>
+        <v>0.439</v>
       </c>
       <c r="Q20" t="n">
-        <v>303</v>
+        <v>321</v>
       </c>
       <c r="R20" t="n">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="S20" t="n">
         <v>22</v>
@@ -2451,7 +2451,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>OBCL LIMITED</t>
+          <t>OBCL LIMITED (FORMERLY KNOWN AS ORISSA BENGAL CARRIER LIMITED)</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2498,10 +2498,10 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>1.541</v>
+        <v>1.607</v>
       </c>
       <c r="Q21" t="n">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="R21" t="inlineStr"/>
       <c r="S21" t="n">
@@ -2593,13 +2593,13 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>0.131</v>
+        <v>0.134</v>
       </c>
       <c r="Q22" t="n">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="R22" t="n">
-        <v>24.7</v>
+        <v>24.1</v>
       </c>
       <c r="S22" t="n">
         <v>12</v>
@@ -2690,13 +2690,13 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="Q23" t="n">
-        <v>347490</v>
+        <v>358204</v>
       </c>
       <c r="R23" t="n">
-        <v>19.1</v>
+        <v>19.7</v>
       </c>
       <c r="S23" t="n">
         <v>7</v>
@@ -2735,12 +2735,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AVONMORE</t>
+          <t>MANINFRA</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>AVONMORE CAPITAL &amp; MANAGEMENT SERVICES LIMITED</t>
+          <t>MAN INFRACONSTRUCTION LIMITED</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -2752,88 +2752,92 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F24" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="G24" t="n">
         <v>20</v>
       </c>
       <c r="H24" t="n">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>13.68</v>
+        <v>115.46</v>
       </c>
       <c r="J24" t="n">
-        <v>12.28</v>
+        <v>105.19</v>
       </c>
       <c r="K24" t="n">
-        <v>11.4</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="L24" t="n">
-        <v>69.12</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="M24" t="n">
-        <v>1.33</v>
+        <v>2.63</v>
       </c>
       <c r="N24" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>26-08-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>0.344</v>
+        <v>0.054</v>
       </c>
       <c r="Q24" t="n">
-        <v>387</v>
+        <v>4906</v>
       </c>
       <c r="R24" t="n">
-        <v>1247</v>
+        <v>32</v>
       </c>
       <c r="S24" t="n">
-        <v>-61</v>
-      </c>
-      <c r="T24" t="inlineStr"/>
+        <v>-25</v>
+      </c>
+      <c r="T24" t="n">
+        <v>71</v>
+      </c>
       <c r="U24" t="n">
-        <v>-98</v>
+        <v>-11</v>
       </c>
       <c r="V24" t="n">
-        <v>0.01</v>
+        <v>1.48</v>
       </c>
       <c r="W24" t="n">
-        <v>2.46</v>
+        <v>10.7</v>
       </c>
       <c r="X24" t="n">
-        <v>0.44</v>
+        <v>0</v>
       </c>
       <c r="Y24" t="b">
         <v>1</v>
       </c>
-      <c r="Z24" t="inlineStr"/>
+      <c r="Z24" t="n">
+        <v>69</v>
+      </c>
       <c r="AA24" t="n">
-        <v>11</v>
+        <v>105</v>
       </c>
       <c r="AB24" t="n">
-        <v>13.57</v>
+        <v>112.45</v>
       </c>
       <c r="AC24" t="n">
-        <v>-8.6</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MANINFRA</t>
+          <t>AVONMORE</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>MAN INFRACONSTRUCTION LIMITED</t>
+          <t>AVONMORE CAPITAL &amp; MANAGEMENT SERVICES LIMITED</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -2845,81 +2849,77 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F25" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="G25" t="n">
         <v>20</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="I25" t="n">
-        <v>115.46</v>
+        <v>13.68</v>
       </c>
       <c r="J25" t="n">
-        <v>105.19</v>
+        <v>12.31</v>
       </c>
       <c r="K25" t="n">
-        <v>9.800000000000001</v>
+        <v>11.1</v>
       </c>
       <c r="L25" t="n">
-        <v>67.15000000000001</v>
+        <v>69.12</v>
       </c>
       <c r="M25" t="n">
-        <v>2.63</v>
+        <v>1.35</v>
       </c>
       <c r="N25" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>27-08-2026</t>
         </is>
       </c>
       <c r="P25" t="n">
-        <v>0.056</v>
+        <v>0.343</v>
       </c>
       <c r="Q25" t="n">
-        <v>4657</v>
+        <v>394</v>
       </c>
       <c r="R25" t="n">
-        <v>30.4</v>
+        <v>1272</v>
       </c>
       <c r="S25" t="n">
-        <v>-25</v>
-      </c>
-      <c r="T25" t="n">
-        <v>71</v>
-      </c>
+        <v>-61</v>
+      </c>
+      <c r="T25" t="inlineStr"/>
       <c r="U25" t="n">
-        <v>-11</v>
+        <v>-98</v>
       </c>
       <c r="V25" t="n">
-        <v>1.48</v>
+        <v>0.01</v>
       </c>
       <c r="W25" t="n">
-        <v>10.7</v>
+        <v>2.46</v>
       </c>
       <c r="X25" t="n">
-        <v>0</v>
+        <v>0.44</v>
       </c>
       <c r="Y25" t="b">
         <v>1</v>
       </c>
-      <c r="Z25" t="n">
-        <v>69</v>
-      </c>
+      <c r="Z25" t="inlineStr"/>
       <c r="AA25" t="n">
-        <v>105</v>
+        <v>11</v>
       </c>
       <c r="AB25" t="n">
-        <v>112.45</v>
+        <v>13.57</v>
       </c>
       <c r="AC25" t="n">
-        <v>3.8</v>
+        <v>-8.6</v>
       </c>
     </row>
     <row r="26">
@@ -2977,13 +2977,13 @@
         </is>
       </c>
       <c r="P26" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="Q26" t="n">
-        <v>5177</v>
+        <v>5144</v>
       </c>
       <c r="R26" t="n">
-        <v>41.5</v>
+        <v>41.2</v>
       </c>
       <c r="S26" t="n">
         <v>0</v>
@@ -3022,12 +3022,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>GOKUL</t>
+          <t>BAJAJHCARE</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>GOKUL REFOILS AND SOLVENT LIMITED</t>
+          <t>BAJAJ HEALTHCARE LIMITED</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3039,92 +3039,92 @@
         </is>
       </c>
       <c r="E27" t="n">
+        <v>22</v>
+      </c>
+      <c r="F27" t="n">
+        <v>21</v>
+      </c>
+      <c r="G27" t="n">
+        <v>5</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>320.9</v>
+      </c>
+      <c r="J27" t="n">
+        <v>297.3</v>
+      </c>
+      <c r="K27" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="L27" t="n">
+        <v>67.69</v>
+      </c>
+      <c r="M27" t="n">
+        <v>2.97</v>
+      </c>
+      <c r="N27" t="n">
+        <v>1</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>12-06-2026</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>0.274</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>1082</v>
+      </c>
+      <c r="R27" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="S27" t="n">
+        <v>12</v>
+      </c>
+      <c r="T27" t="n">
+        <v>29</v>
+      </c>
+      <c r="U27" t="n">
         <v>20</v>
       </c>
-      <c r="F27" t="n">
-        <v>8</v>
-      </c>
-      <c r="G27" t="n">
-        <v>25</v>
-      </c>
-      <c r="H27" t="n">
-        <v>-5</v>
-      </c>
-      <c r="I27" t="n">
-        <v>43.09</v>
-      </c>
-      <c r="J27" t="n">
-        <v>43.02</v>
-      </c>
-      <c r="K27" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="L27" t="n">
-        <v>71.79000000000001</v>
-      </c>
-      <c r="M27" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="N27" t="n">
-        <v>21</v>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>25-08-2026</t>
-        </is>
-      </c>
-      <c r="P27" t="n">
-        <v>0.237</v>
-      </c>
-      <c r="Q27" t="n">
-        <v>427</v>
-      </c>
-      <c r="R27" t="n">
-        <v>106</v>
-      </c>
-      <c r="S27" t="n">
-        <v>246</v>
-      </c>
-      <c r="T27" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="U27" t="n">
-        <v>10</v>
-      </c>
       <c r="V27" t="n">
-        <v>0.14</v>
+        <v>4.07</v>
       </c>
       <c r="W27" t="n">
-        <v>2.16</v>
+        <v>11.5</v>
       </c>
       <c r="X27" t="n">
-        <v>0</v>
+        <v>0.47</v>
       </c>
       <c r="Y27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z27" t="n">
-        <v>4.21</v>
+        <v>17</v>
       </c>
       <c r="AA27" t="n">
-        <v>40.73</v>
+        <v>333.67</v>
       </c>
       <c r="AB27" t="n">
-        <v>39.65</v>
+        <v>350.41</v>
       </c>
       <c r="AC27" t="n">
-        <v>8.9</v>
+        <v>-9</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>BAJAJHCARE</t>
+          <t>GOKUL</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>BAJAJ HEALTHCARE LIMITED</t>
+          <t>GOKUL REFOILS AND SOLVENT LIMITED</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3136,81 +3136,81 @@
         </is>
       </c>
       <c r="E28" t="n">
+        <v>20</v>
+      </c>
+      <c r="F28" t="n">
+        <v>8</v>
+      </c>
+      <c r="G28" t="n">
+        <v>25</v>
+      </c>
+      <c r="H28" t="n">
+        <v>-5</v>
+      </c>
+      <c r="I28" t="n">
+        <v>43.09</v>
+      </c>
+      <c r="J28" t="n">
+        <v>43.04</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L28" t="n">
+        <v>71.79000000000001</v>
+      </c>
+      <c r="M28" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="N28" t="n">
         <v>22</v>
       </c>
-      <c r="F28" t="n">
-        <v>21</v>
-      </c>
-      <c r="G28" t="n">
-        <v>5</v>
-      </c>
-      <c r="H28" t="n">
-        <v>0</v>
-      </c>
-      <c r="I28" t="n">
-        <v>320.9</v>
-      </c>
-      <c r="J28" t="n">
-        <v>297.3</v>
-      </c>
-      <c r="K28" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="L28" t="n">
-        <v>67.69</v>
-      </c>
-      <c r="M28" t="n">
-        <v>2.97</v>
-      </c>
-      <c r="N28" t="n">
-        <v>1</v>
-      </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>12-06-2026</t>
+          <t>26-08-2026</t>
         </is>
       </c>
       <c r="P28" t="n">
-        <v>0.274</v>
+        <v>0.24</v>
       </c>
       <c r="Q28" t="n">
-        <v>1082</v>
+        <v>425</v>
       </c>
       <c r="R28" t="n">
-        <v>19.2</v>
+        <v>105</v>
       </c>
       <c r="S28" t="n">
-        <v>12</v>
+        <v>246</v>
       </c>
       <c r="T28" t="n">
-        <v>29</v>
+        <v>0.91</v>
       </c>
       <c r="U28" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="V28" t="n">
-        <v>4.07</v>
+        <v>0.14</v>
       </c>
       <c r="W28" t="n">
-        <v>11.5</v>
+        <v>2.16</v>
       </c>
       <c r="X28" t="n">
-        <v>0.47</v>
+        <v>0</v>
       </c>
       <c r="Y28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z28" t="n">
-        <v>17</v>
+        <v>4.21</v>
       </c>
       <c r="AA28" t="n">
-        <v>333.67</v>
+        <v>40.73</v>
       </c>
       <c r="AB28" t="n">
-        <v>350.41</v>
+        <v>39.65</v>
       </c>
       <c r="AC28" t="n">
-        <v>-9</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="29">
@@ -3268,13 +3268,13 @@
         </is>
       </c>
       <c r="P29" t="n">
-        <v>1.276</v>
+        <v>1.252</v>
       </c>
       <c r="Q29" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="R29" t="n">
-        <v>75.40000000000001</v>
+        <v>77.3</v>
       </c>
       <c r="S29" t="n">
         <v>-1</v>
@@ -3368,10 +3368,10 @@
         <v>0.011</v>
       </c>
       <c r="Q30" t="n">
-        <v>2265</v>
+        <v>2312</v>
       </c>
       <c r="R30" t="n">
-        <v>52</v>
+        <v>53.1</v>
       </c>
       <c r="S30" t="n">
         <v>20</v>
@@ -3415,7 +3415,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Ganesh Consumer Products Limited</t>
+          <t>GANESH CONSUMER PRODUCTS LIMITED</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -3442,33 +3442,33 @@
         <v>163.49</v>
       </c>
       <c r="J31" t="n">
-        <v>204.13</v>
+        <v>201.21</v>
       </c>
       <c r="K31" t="n">
-        <v>-19.9</v>
+        <v>-18.7</v>
       </c>
       <c r="L31" t="n">
         <v>64.08</v>
       </c>
       <c r="M31" t="n">
-        <v>7.57</v>
+        <v>8.07</v>
       </c>
       <c r="N31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>30-06-2026</t>
+          <t>25-08-2026</t>
         </is>
       </c>
       <c r="P31" t="n">
-        <v>1.144</v>
+        <v>1.13</v>
       </c>
       <c r="Q31" t="n">
-        <v>662</v>
+        <v>714</v>
       </c>
       <c r="R31" t="n">
-        <v>14.6</v>
+        <v>15.7</v>
       </c>
       <c r="S31" t="n">
         <v>-1</v>
@@ -3562,10 +3562,10 @@
         <v>0.126</v>
       </c>
       <c r="Q32" t="n">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="R32" t="n">
-        <v>13.9</v>
+        <v>14</v>
       </c>
       <c r="S32" t="n">
         <v>61</v>
@@ -3602,12 +3602,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ARSSBL</t>
+          <t>PKTEA</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Anand Rathi Share and Stock Brokers Limited</t>
+          <t>THE PERIA KARAMALAI TEA &amp; PRODUCE COMPANY LIMITED</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -3619,92 +3619,90 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F33" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="G33" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>517.05</v>
+        <v>751.85</v>
       </c>
       <c r="J33" t="n">
-        <v>545.03</v>
+        <v>717.77</v>
       </c>
       <c r="K33" t="n">
-        <v>-5.1</v>
+        <v>4.7</v>
       </c>
       <c r="L33" t="n">
-        <v>69.90000000000001</v>
+        <v>61.71</v>
       </c>
       <c r="M33" t="n">
-        <v>1.09</v>
+        <v>1.61</v>
       </c>
       <c r="N33" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>16-06-2026</t>
+          <t>20-08-2026</t>
         </is>
       </c>
       <c r="P33" t="n">
-        <v>0.033</v>
+        <v>0.6879999999999999</v>
       </c>
       <c r="Q33" t="n">
-        <v>3260</v>
-      </c>
-      <c r="R33" t="n">
-        <v>22.1</v>
-      </c>
+        <v>234</v>
+      </c>
+      <c r="R33" t="inlineStr"/>
       <c r="S33" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="T33" t="n">
-        <v>97</v>
+        <v>11.91</v>
       </c>
       <c r="U33" t="n">
-        <v>53</v>
+        <v>-184</v>
       </c>
       <c r="V33" t="n">
-        <v>3.73</v>
+        <v>31.98</v>
       </c>
       <c r="W33" t="n">
-        <v>19.8</v>
+        <v>0.27</v>
       </c>
       <c r="X33" t="n">
-        <v>0.62</v>
+        <v>0.1</v>
       </c>
       <c r="Y33" t="b">
         <v>1</v>
       </c>
       <c r="Z33" t="n">
-        <v>40</v>
+        <v>57.93</v>
       </c>
       <c r="AA33" t="n">
-        <v>531.78</v>
+        <v>731.62</v>
       </c>
       <c r="AB33" t="n">
-        <v>563.13</v>
+        <v>760.35</v>
       </c>
       <c r="AC33" t="n">
-        <v>-1.6</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>PKTEA</t>
+          <t>ARSSBL</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>THE PERIA KARAMALAI TEA &amp; PRODUCE COMPANY LIMITED</t>
+          <t>Anand Rathi Share and Stock Brokers Limited</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -3716,79 +3714,81 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F34" t="n">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="G34" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H34" t="n">
         <v>0</v>
       </c>
       <c r="I34" t="n">
-        <v>751.85</v>
+        <v>517.05</v>
       </c>
       <c r="J34" t="n">
-        <v>717.77</v>
+        <v>545.03</v>
       </c>
       <c r="K34" t="n">
-        <v>4.7</v>
+        <v>-5.1</v>
       </c>
       <c r="L34" t="n">
-        <v>61.71</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="M34" t="n">
-        <v>1.61</v>
+        <v>1.09</v>
       </c>
       <c r="N34" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>20-08-2026</t>
+          <t>16-06-2026</t>
         </is>
       </c>
       <c r="P34" t="n">
-        <v>0.6909999999999999</v>
+        <v>0.033</v>
       </c>
       <c r="Q34" t="n">
-        <v>233</v>
-      </c>
-      <c r="R34" t="inlineStr"/>
+        <v>3261</v>
+      </c>
+      <c r="R34" t="n">
+        <v>22.1</v>
+      </c>
       <c r="S34" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="T34" t="n">
-        <v>11.91</v>
+        <v>97</v>
       </c>
       <c r="U34" t="n">
-        <v>-184</v>
+        <v>53</v>
       </c>
       <c r="V34" t="n">
-        <v>31.98</v>
+        <v>3.73</v>
       </c>
       <c r="W34" t="n">
-        <v>0.27</v>
+        <v>19.8</v>
       </c>
       <c r="X34" t="n">
-        <v>0.1</v>
+        <v>0.62</v>
       </c>
       <c r="Y34" t="b">
         <v>1</v>
       </c>
       <c r="Z34" t="n">
-        <v>57.93</v>
+        <v>40</v>
       </c>
       <c r="AA34" t="n">
-        <v>731.62</v>
+        <v>531.78</v>
       </c>
       <c r="AB34" t="n">
-        <v>760.35</v>
+        <v>563.13</v>
       </c>
       <c r="AC34" t="n">
-        <v>-3</v>
+        <v>-1.6</v>
       </c>
     </row>
     <row r="35">
@@ -3846,13 +3846,13 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>0.32</v>
+        <v>0.322</v>
       </c>
       <c r="Q35" t="n">
-        <v>2303</v>
+        <v>2287</v>
       </c>
       <c r="R35" t="n">
-        <v>19.8</v>
+        <v>19.6</v>
       </c>
       <c r="S35" t="n">
         <v>18</v>
@@ -3891,16 +3891,16 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>EUROPRATIK</t>
+          <t>VIVIANA</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Euro Pratik Sales Limited</t>
+          <t>VIVIANA POWER TECH LIMITED</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -3908,96 +3908,94 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F36" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="G36" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H36" t="n">
         <v>0</v>
       </c>
       <c r="I36" t="n">
-        <v>254.05</v>
+        <v>729.3</v>
       </c>
       <c r="J36" t="n">
-        <v>259.44</v>
+        <v>815.16</v>
       </c>
       <c r="K36" t="n">
-        <v>-2.1</v>
+        <v>-10.5</v>
       </c>
       <c r="L36" t="n">
-        <v>70.09</v>
+        <v>73.2</v>
       </c>
       <c r="M36" t="n">
-        <v>29.05</v>
+        <v>1.24</v>
       </c>
       <c r="N36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>29-05-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="P36" t="n">
-        <v>1.118</v>
+        <v>0.169</v>
       </c>
       <c r="Q36" t="n">
-        <v>2598</v>
+        <v>732</v>
       </c>
       <c r="R36" t="n">
-        <v>45.2</v>
+        <v>13.3</v>
       </c>
       <c r="S36" t="n">
-        <v>-3</v>
+        <v>185</v>
       </c>
       <c r="T36" t="n">
-        <v>11</v>
+        <v>11.55</v>
       </c>
       <c r="U36" t="n">
-        <v>3</v>
+        <v>204</v>
       </c>
       <c r="V36" t="n">
-        <v>1.05</v>
+        <v>6.84</v>
       </c>
       <c r="W36" t="n">
-        <v>29.6</v>
+        <v>50.7</v>
       </c>
       <c r="X36" t="n">
-        <v>0.03</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="Y36" t="b">
         <v>1</v>
       </c>
       <c r="Z36" t="n">
-        <v>24</v>
+        <v>16.07</v>
       </c>
       <c r="AA36" t="n">
-        <v>294.76</v>
-      </c>
-      <c r="AB36" t="n">
-        <v>278.19</v>
-      </c>
+        <v>751.4</v>
+      </c>
+      <c r="AB36" t="inlineStr"/>
       <c r="AC36" t="n">
-        <v>-1.8</v>
+        <v>-19.8</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>VIVIANA</t>
+          <t>TRUALT</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>VIVIANA POWER TECH LIMITED</t>
+          <t>TRUALT BIOENERGY LIMITED</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -4005,191 +4003,183 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F37" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="G37" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H37" t="n">
         <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>729.3</v>
+        <v>433.85</v>
       </c>
       <c r="J37" t="n">
-        <v>815.16</v>
+        <v>474.82</v>
       </c>
       <c r="K37" t="n">
-        <v>-10.5</v>
+        <v>-8.6</v>
       </c>
       <c r="L37" t="n">
-        <v>73.2</v>
+        <v>70.55</v>
       </c>
       <c r="M37" t="n">
-        <v>1.24</v>
+        <v>10.22</v>
       </c>
       <c r="N37" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>12-08-2026</t>
         </is>
       </c>
       <c r="P37" t="n">
-        <v>0.168</v>
+        <v>0.275</v>
       </c>
       <c r="Q37" t="n">
-        <v>738</v>
+        <v>3719</v>
       </c>
       <c r="R37" t="n">
-        <v>13.4</v>
+        <v>26</v>
       </c>
       <c r="S37" t="n">
-        <v>185</v>
+        <v>2</v>
       </c>
       <c r="T37" t="n">
-        <v>11.55</v>
+        <v>127</v>
       </c>
       <c r="U37" t="n">
-        <v>204</v>
+        <v>-14</v>
       </c>
       <c r="V37" t="n">
-        <v>6.84</v>
+        <v>6.41</v>
       </c>
       <c r="W37" t="n">
-        <v>50.7</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="X37" t="n">
-        <v>0.8100000000000001</v>
+        <v>1.05</v>
       </c>
       <c r="Y37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z37" t="n">
-        <v>16.07</v>
+        <v>21</v>
       </c>
       <c r="AA37" t="n">
-        <v>751.4</v>
-      </c>
-      <c r="AB37" t="inlineStr"/>
+        <v>451.75</v>
+      </c>
+      <c r="AB37" t="n">
+        <v>434.25</v>
+      </c>
       <c r="AC37" t="n">
-        <v>-19.8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TRUALT</t>
+          <t>HEXAGON</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>TRUALT BIOENERGY LIMITED</t>
+          <t>HEXAGON NUTRITION LIMITED</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Watchlist</t>
+          <t>Fundamental Watch</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="F38" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G38" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H38" t="n">
         <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>433.85</v>
+        <v>69.16</v>
       </c>
       <c r="J38" t="n">
-        <v>474.82</v>
+        <v>64.04000000000001</v>
       </c>
       <c r="K38" t="n">
-        <v>-8.6</v>
+        <v>8</v>
       </c>
       <c r="L38" t="n">
-        <v>70.55</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="M38" t="n">
-        <v>10.22</v>
+        <v>0.31</v>
       </c>
       <c r="N38" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>12-08-2026</t>
+          <t>17-08-2026</t>
         </is>
       </c>
       <c r="P38" t="n">
-        <v>0.274</v>
+        <v>0.036</v>
       </c>
       <c r="Q38" t="n">
-        <v>3725</v>
+        <v>852</v>
       </c>
       <c r="R38" t="n">
-        <v>26.1</v>
-      </c>
-      <c r="S38" t="n">
-        <v>2</v>
-      </c>
+        <v>20.4</v>
+      </c>
+      <c r="S38" t="inlineStr"/>
       <c r="T38" t="n">
-        <v>127</v>
-      </c>
-      <c r="U38" t="n">
-        <v>-14</v>
-      </c>
+        <v>12.31</v>
+      </c>
+      <c r="U38" t="inlineStr"/>
       <c r="V38" t="n">
-        <v>6.41</v>
-      </c>
-      <c r="W38" t="n">
-        <v>9.890000000000001</v>
-      </c>
+        <v>0.8</v>
+      </c>
+      <c r="W38" t="inlineStr"/>
       <c r="X38" t="n">
-        <v>1.05</v>
+        <v>0.11</v>
       </c>
       <c r="Y38" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z38" t="n">
-        <v>21</v>
+        <v>12.14</v>
       </c>
       <c r="AA38" t="n">
-        <v>451.75</v>
-      </c>
-      <c r="AB38" t="n">
-        <v>434.25</v>
-      </c>
-      <c r="AC38" t="n">
-        <v>6</v>
-      </c>
+        <v>65.86</v>
+      </c>
+      <c r="AB38" t="inlineStr"/>
+      <c r="AC38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>HEXAGON</t>
+          <t>BMWVENTLTD</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>HEXAGON NUTRITION LIMITED</t>
+          <t>BMW VENTURES LIMITED</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -4197,72 +4187,82 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F39" t="n">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="G39" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="I39" t="n">
-        <v>69.16</v>
+        <v>56.95</v>
       </c>
       <c r="J39" t="n">
-        <v>64.04000000000001</v>
+        <v>60.15</v>
       </c>
       <c r="K39" t="n">
-        <v>8</v>
+        <v>-5.3</v>
       </c>
       <c r="L39" t="n">
-        <v>64.29000000000001</v>
+        <v>73.01000000000001</v>
       </c>
       <c r="M39" t="n">
-        <v>0.31</v>
+        <v>0.9</v>
       </c>
       <c r="N39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>17-08-2026</t>
+          <t>06-08-2026</t>
         </is>
       </c>
       <c r="P39" t="n">
-        <v>0.037</v>
+        <v>0.183</v>
       </c>
       <c r="Q39" t="n">
-        <v>849</v>
+        <v>492</v>
       </c>
       <c r="R39" t="n">
-        <v>20.3</v>
-      </c>
-      <c r="S39" t="inlineStr"/>
+        <v>12.3</v>
+      </c>
+      <c r="S39" t="n">
+        <v>19</v>
+      </c>
       <c r="T39" t="n">
-        <v>12.31</v>
-      </c>
-      <c r="U39" t="inlineStr"/>
+        <v>21</v>
+      </c>
+      <c r="U39" t="n">
+        <v>20</v>
+      </c>
       <c r="V39" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="W39" t="inlineStr"/>
+        <v>1.22</v>
+      </c>
+      <c r="W39" t="n">
+        <v>12</v>
+      </c>
       <c r="X39" t="n">
-        <v>0.11</v>
+        <v>0.58</v>
       </c>
       <c r="Y39" t="b">
         <v>1</v>
       </c>
       <c r="Z39" t="n">
-        <v>12.14</v>
+        <v>3.4</v>
       </c>
       <c r="AA39" t="n">
-        <v>65.86</v>
-      </c>
-      <c r="AB39" t="inlineStr"/>
-      <c r="AC39" t="inlineStr"/>
+        <v>57.94</v>
+      </c>
+      <c r="AB39" t="n">
+        <v>59.37</v>
+      </c>
+      <c r="AC39" t="n">
+        <v>-3.6</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4319,13 +4319,13 @@
         </is>
       </c>
       <c r="P40" t="n">
-        <v>0.098</v>
+        <v>0.097</v>
       </c>
       <c r="Q40" t="n">
-        <v>1507</v>
+        <v>1526</v>
       </c>
       <c r="R40" t="n">
-        <v>13.6</v>
+        <v>13.8</v>
       </c>
       <c r="S40" t="n">
         <v>6</v>
@@ -4364,16 +4364,16 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>BMWVENTLTD</t>
+          <t>GRMOVER</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>BMW VENTURES LIMITED</t>
+          <t>GRM OVERSEAS LIMITED</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -4381,92 +4381,92 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F41" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="G41" t="n">
         <v>0</v>
       </c>
       <c r="H41" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="I41" t="n">
-        <v>56.95</v>
+        <v>87.76000000000001</v>
       </c>
       <c r="J41" t="n">
-        <v>60.15</v>
+        <v>95.54000000000001</v>
       </c>
       <c r="K41" t="n">
-        <v>-5.3</v>
+        <v>-8.1</v>
       </c>
       <c r="L41" t="n">
-        <v>73.01000000000001</v>
+        <v>71.72</v>
       </c>
       <c r="M41" t="n">
+        <v>10.87</v>
+      </c>
+      <c r="N41" t="n">
+        <v>6</v>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>24-06-2026</t>
+        </is>
+      </c>
+      <c r="P41" t="n">
+        <v>0.601</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>1808</v>
+      </c>
+      <c r="R41" t="n">
+        <v>32.6</v>
+      </c>
+      <c r="S41" t="n">
+        <v>39</v>
+      </c>
+      <c r="T41" t="n">
+        <v>31</v>
+      </c>
+      <c r="U41" t="n">
+        <v>8</v>
+      </c>
+      <c r="V41" t="n">
         <v>0.9</v>
       </c>
-      <c r="N41" t="n">
-        <v>2</v>
-      </c>
-      <c r="O41" t="inlineStr">
-        <is>
-          <t>06-08-2026</t>
-        </is>
-      </c>
-      <c r="P41" t="n">
-        <v>0.181</v>
-      </c>
-      <c r="Q41" t="n">
-        <v>496</v>
-      </c>
-      <c r="R41" t="n">
-        <v>12.4</v>
-      </c>
-      <c r="S41" t="n">
-        <v>19</v>
-      </c>
-      <c r="T41" t="n">
-        <v>21</v>
-      </c>
-      <c r="U41" t="n">
-        <v>20</v>
-      </c>
-      <c r="V41" t="n">
-        <v>1.22</v>
-      </c>
       <c r="W41" t="n">
-        <v>12</v>
+        <v>11.3</v>
       </c>
       <c r="X41" t="n">
-        <v>0.58</v>
+        <v>0.67</v>
       </c>
       <c r="Y41" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z41" t="n">
-        <v>3.4</v>
+        <v>9</v>
       </c>
       <c r="AA41" t="n">
-        <v>57.94</v>
+        <v>91.67</v>
       </c>
       <c r="AB41" t="n">
-        <v>59.37</v>
+        <v>193.41</v>
       </c>
       <c r="AC41" t="n">
-        <v>-3.6</v>
+        <v>-45.6</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>GRMOVER</t>
+          <t>EUROPRATIK</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>GRM OVERSEAS LIMITED</t>
+          <t>Euro Pratik Sales Limited</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -4478,81 +4478,81 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F42" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G42" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H42" t="n">
         <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>87.76000000000001</v>
+        <v>254.05</v>
       </c>
       <c r="J42" t="n">
-        <v>95.54000000000001</v>
+        <v>257.65</v>
       </c>
       <c r="K42" t="n">
-        <v>-8.1</v>
+        <v>-1.4</v>
       </c>
       <c r="L42" t="n">
-        <v>71.72</v>
+        <v>70.09</v>
       </c>
       <c r="M42" t="n">
-        <v>10.87</v>
+        <v>1.64</v>
       </c>
       <c r="N42" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>24-06-2026</t>
+          <t>29-05-2026</t>
         </is>
       </c>
       <c r="P42" t="n">
-        <v>0.598</v>
+        <v>0.062</v>
       </c>
       <c r="Q42" t="n">
-        <v>1818</v>
+        <v>2633</v>
       </c>
       <c r="R42" t="n">
-        <v>32.8</v>
+        <v>45.8</v>
       </c>
       <c r="S42" t="n">
-        <v>39</v>
+        <v>-3</v>
       </c>
       <c r="T42" t="n">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="U42" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="V42" t="n">
-        <v>0.9</v>
+        <v>1.05</v>
       </c>
       <c r="W42" t="n">
-        <v>11.3</v>
+        <v>29.6</v>
       </c>
       <c r="X42" t="n">
-        <v>0.67</v>
+        <v>0.03</v>
       </c>
       <c r="Y42" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z42" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="AA42" t="n">
-        <v>91.67</v>
+        <v>294.76</v>
       </c>
       <c r="AB42" t="n">
-        <v>193.41</v>
+        <v>278.19</v>
       </c>
       <c r="AC42" t="n">
-        <v>-45.6</v>
+        <v>-1.8</v>
       </c>
     </row>
     <row r="43">
@@ -4610,13 +4610,13 @@
         </is>
       </c>
       <c r="P43" t="n">
-        <v>0.202</v>
+        <v>0.201</v>
       </c>
       <c r="Q43" t="n">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="R43" t="n">
-        <v>25.4</v>
+        <v>25.5</v>
       </c>
       <c r="S43" t="n">
         <v>21</v>
@@ -4804,10 +4804,10 @@
         </is>
       </c>
       <c r="P45" t="n">
-        <v>0.082</v>
+        <v>0.083</v>
       </c>
       <c r="Q45" t="n">
-        <v>1564</v>
+        <v>1562</v>
       </c>
       <c r="R45" t="n">
         <v>19.8</v>
@@ -4901,13 +4901,13 @@
         </is>
       </c>
       <c r="P46" t="n">
-        <v>0.276</v>
+        <v>0.28</v>
       </c>
       <c r="Q46" t="n">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="R46" t="n">
-        <v>16.8</v>
+        <v>16.6</v>
       </c>
       <c r="S46" t="n">
         <v>16</v>
@@ -4998,13 +4998,13 @@
         </is>
       </c>
       <c r="P47" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="Q47" t="n">
-        <v>885</v>
+        <v>873</v>
       </c>
       <c r="R47" t="n">
-        <v>24.1</v>
+        <v>23.8</v>
       </c>
       <c r="S47" t="n">
         <v>9</v>
@@ -5095,13 +5095,13 @@
         </is>
       </c>
       <c r="P48" t="n">
-        <v>0.039</v>
+        <v>0.038</v>
       </c>
       <c r="Q48" t="n">
-        <v>803</v>
+        <v>812</v>
       </c>
       <c r="R48" t="n">
-        <v>7.9</v>
+        <v>7.98</v>
       </c>
       <c r="S48" t="n">
         <v>7</v>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Gandhar Oil Refinery (India) Limited</t>
+          <t>GANDHAR OIL REFINERY (INDIA) LIMITED</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -5259,19 +5259,19 @@
         <v>95.20999999999999</v>
       </c>
       <c r="D3" t="n">
-        <v>55.67</v>
+        <v>55.78</v>
       </c>
       <c r="E3" t="n">
-        <v>71</v>
+        <v>70.7</v>
       </c>
       <c r="F3" t="n">
         <v>67.45999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>6.76</v>
+        <v>6.19</v>
       </c>
       <c r="H3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -5492,70 +5492,70 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>CHEMBONDCH</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PNGS Reva Diamond Jewellery Limited</t>
+          <t>CHEMBOND CHEMICALS LIMITED</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>542.9</v>
+        <v>269.84</v>
       </c>
       <c r="D10" t="n">
-        <v>390.61</v>
+        <v>243.52</v>
       </c>
       <c r="E10" t="n">
-        <v>39</v>
+        <v>10.8</v>
       </c>
       <c r="F10" t="n">
-        <v>63.09</v>
+        <v>67.65000000000001</v>
       </c>
       <c r="G10" t="n">
-        <v>8.02</v>
+        <v>1.11</v>
       </c>
       <c r="H10" t="n">
         <v>3</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>25-08-2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CHEMBONDCH</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CHEMBOND CHEMICALS LIMITED</t>
+          <t>PNGS Reva Diamond Jewellery Limited</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>269.84</v>
+        <v>542.9</v>
       </c>
       <c r="D11" t="n">
-        <v>243.52</v>
+        <v>390.61</v>
       </c>
       <c r="E11" t="n">
-        <v>10.8</v>
+        <v>39</v>
       </c>
       <c r="F11" t="n">
-        <v>67.65000000000001</v>
+        <v>63.09</v>
       </c>
       <c r="G11" t="n">
-        <v>1.11</v>
+        <v>8.02</v>
       </c>
       <c r="H11" t="n">
         <v>3</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>25-08-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
     </row>
@@ -5882,7 +5882,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>OBCL LIMITED</t>
+          <t>OBCL LIMITED (FORMERLY KNOWN AS ORISSA BENGAL CARRIER LIMITED)</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -5982,70 +5982,70 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AVONMORE</t>
+          <t>MANINFRA</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>AVONMORE CAPITAL &amp; MANAGEMENT SERVICES LIMITED</t>
+          <t>MAN INFRACONSTRUCTION LIMITED</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>13.68</v>
+        <v>115.46</v>
       </c>
       <c r="D24" t="n">
-        <v>12.28</v>
+        <v>105.19</v>
       </c>
       <c r="E24" t="n">
-        <v>11.4</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F24" t="n">
-        <v>69.12</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="G24" t="n">
-        <v>1.33</v>
+        <v>2.63</v>
       </c>
       <c r="H24" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>26-08-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MANINFRA</t>
+          <t>AVONMORE</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>MAN INFRACONSTRUCTION LIMITED</t>
+          <t>AVONMORE CAPITAL &amp; MANAGEMENT SERVICES LIMITED</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>115.46</v>
+        <v>13.68</v>
       </c>
       <c r="D25" t="n">
-        <v>105.19</v>
+        <v>12.31</v>
       </c>
       <c r="E25" t="n">
-        <v>9.800000000000001</v>
+        <v>11.1</v>
       </c>
       <c r="F25" t="n">
-        <v>67.15000000000001</v>
+        <v>69.12</v>
       </c>
       <c r="G25" t="n">
-        <v>2.63</v>
+        <v>1.35</v>
       </c>
       <c r="H25" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>27-08-2026</t>
         </is>
       </c>
     </row>
@@ -6087,70 +6087,70 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>GOKUL</t>
+          <t>BAJAJHCARE</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>GOKUL REFOILS AND SOLVENT LIMITED</t>
+          <t>BAJAJ HEALTHCARE LIMITED</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>43.09</v>
+        <v>320.9</v>
       </c>
       <c r="D27" t="n">
-        <v>43.02</v>
+        <v>297.3</v>
       </c>
       <c r="E27" t="n">
-        <v>0.2</v>
+        <v>7.9</v>
       </c>
       <c r="F27" t="n">
-        <v>71.79000000000001</v>
+        <v>67.69</v>
       </c>
       <c r="G27" t="n">
-        <v>1.01</v>
+        <v>2.97</v>
       </c>
       <c r="H27" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>25-08-2026</t>
+          <t>12-06-2026</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>BAJAJHCARE</t>
+          <t>GOKUL</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>BAJAJ HEALTHCARE LIMITED</t>
+          <t>GOKUL REFOILS AND SOLVENT LIMITED</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>320.9</v>
+        <v>43.09</v>
       </c>
       <c r="D28" t="n">
-        <v>297.3</v>
+        <v>43.04</v>
       </c>
       <c r="E28" t="n">
-        <v>7.9</v>
+        <v>0.1</v>
       </c>
       <c r="F28" t="n">
-        <v>67.69</v>
+        <v>71.79000000000001</v>
       </c>
       <c r="G28" t="n">
-        <v>2.97</v>
+        <v>1.02</v>
       </c>
       <c r="H28" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>12-06-2026</t>
+          <t>26-08-2026</t>
         </is>
       </c>
     </row>
@@ -6232,30 +6232,30 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Ganesh Consumer Products Limited</t>
+          <t>GANESH CONSUMER PRODUCTS LIMITED</t>
         </is>
       </c>
       <c r="C31" t="n">
         <v>163.49</v>
       </c>
       <c r="D31" t="n">
-        <v>204.13</v>
+        <v>201.21</v>
       </c>
       <c r="E31" t="n">
-        <v>-19.9</v>
+        <v>-18.7</v>
       </c>
       <c r="F31" t="n">
         <v>64.08</v>
       </c>
       <c r="G31" t="n">
-        <v>7.57</v>
+        <v>8.07</v>
       </c>
       <c r="H31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>30-06-2026</t>
+          <t>25-08-2026</t>
         </is>
       </c>
     </row>
@@ -6297,70 +6297,70 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ARSSBL</t>
+          <t>PKTEA</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Anand Rathi Share and Stock Brokers Limited</t>
+          <t>THE PERIA KARAMALAI TEA &amp; PRODUCE COMPANY LIMITED</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>517.05</v>
+        <v>751.85</v>
       </c>
       <c r="D33" t="n">
-        <v>545.03</v>
+        <v>717.77</v>
       </c>
       <c r="E33" t="n">
-        <v>-5.1</v>
+        <v>4.7</v>
       </c>
       <c r="F33" t="n">
-        <v>69.90000000000001</v>
+        <v>61.71</v>
       </c>
       <c r="G33" t="n">
-        <v>1.09</v>
+        <v>1.61</v>
       </c>
       <c r="H33" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>16-06-2026</t>
+          <t>20-08-2026</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>PKTEA</t>
+          <t>ARSSBL</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>THE PERIA KARAMALAI TEA &amp; PRODUCE COMPANY LIMITED</t>
+          <t>Anand Rathi Share and Stock Brokers Limited</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>751.85</v>
+        <v>517.05</v>
       </c>
       <c r="D34" t="n">
-        <v>717.77</v>
+        <v>545.03</v>
       </c>
       <c r="E34" t="n">
-        <v>4.7</v>
+        <v>-5.1</v>
       </c>
       <c r="F34" t="n">
-        <v>61.71</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="G34" t="n">
-        <v>1.61</v>
+        <v>1.09</v>
       </c>
       <c r="H34" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>20-08-2026</t>
+          <t>16-06-2026</t>
         </is>
       </c>
     </row>
@@ -6402,140 +6402,140 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>EUROPRATIK</t>
+          <t>VIVIANA</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Euro Pratik Sales Limited</t>
+          <t>VIVIANA POWER TECH LIMITED</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>254.05</v>
+        <v>729.3</v>
       </c>
       <c r="D36" t="n">
-        <v>259.44</v>
+        <v>815.16</v>
       </c>
       <c r="E36" t="n">
-        <v>-2.1</v>
+        <v>-10.5</v>
       </c>
       <c r="F36" t="n">
-        <v>70.09</v>
+        <v>73.2</v>
       </c>
       <c r="G36" t="n">
-        <v>29.05</v>
+        <v>1.24</v>
       </c>
       <c r="H36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>29-05-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>VIVIANA</t>
+          <t>TRUALT</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>VIVIANA POWER TECH LIMITED</t>
+          <t>TRUALT BIOENERGY LIMITED</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>729.3</v>
+        <v>433.85</v>
       </c>
       <c r="D37" t="n">
-        <v>815.16</v>
+        <v>474.82</v>
       </c>
       <c r="E37" t="n">
-        <v>-10.5</v>
+        <v>-8.6</v>
       </c>
       <c r="F37" t="n">
-        <v>73.2</v>
+        <v>70.55</v>
       </c>
       <c r="G37" t="n">
-        <v>1.24</v>
+        <v>10.22</v>
       </c>
       <c r="H37" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>12-08-2026</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TRUALT</t>
+          <t>HEXAGON</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>TRUALT BIOENERGY LIMITED</t>
+          <t>HEXAGON NUTRITION LIMITED</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>433.85</v>
+        <v>69.16</v>
       </c>
       <c r="D38" t="n">
-        <v>474.82</v>
+        <v>64.04000000000001</v>
       </c>
       <c r="E38" t="n">
-        <v>-8.6</v>
+        <v>8</v>
       </c>
       <c r="F38" t="n">
-        <v>70.55</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="G38" t="n">
-        <v>10.22</v>
+        <v>0.31</v>
       </c>
       <c r="H38" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>12-08-2026</t>
+          <t>17-08-2026</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>HEXAGON</t>
+          <t>BMWVENTLTD</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>HEXAGON NUTRITION LIMITED</t>
+          <t>BMW VENTURES LIMITED</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>69.16</v>
+        <v>56.95</v>
       </c>
       <c r="D39" t="n">
-        <v>64.04000000000001</v>
+        <v>60.15</v>
       </c>
       <c r="E39" t="n">
-        <v>8</v>
+        <v>-5.3</v>
       </c>
       <c r="F39" t="n">
-        <v>64.29000000000001</v>
+        <v>73.01000000000001</v>
       </c>
       <c r="G39" t="n">
-        <v>0.31</v>
+        <v>0.9</v>
       </c>
       <c r="H39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>17-08-2026</t>
+          <t>06-08-2026</t>
         </is>
       </c>
     </row>
@@ -6577,70 +6577,70 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>BMWVENTLTD</t>
+          <t>GRMOVER</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>BMW VENTURES LIMITED</t>
+          <t>GRM OVERSEAS LIMITED</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>56.95</v>
+        <v>87.76000000000001</v>
       </c>
       <c r="D41" t="n">
-        <v>60.15</v>
+        <v>95.54000000000001</v>
       </c>
       <c r="E41" t="n">
-        <v>-5.3</v>
+        <v>-8.1</v>
       </c>
       <c r="F41" t="n">
-        <v>73.01000000000001</v>
+        <v>71.72</v>
       </c>
       <c r="G41" t="n">
-        <v>0.9</v>
+        <v>10.87</v>
       </c>
       <c r="H41" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>06-08-2026</t>
+          <t>24-06-2026</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>GRMOVER</t>
+          <t>EUROPRATIK</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>GRM OVERSEAS LIMITED</t>
+          <t>Euro Pratik Sales Limited</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>87.76000000000001</v>
+        <v>254.05</v>
       </c>
       <c r="D42" t="n">
-        <v>95.54000000000001</v>
+        <v>257.65</v>
       </c>
       <c r="E42" t="n">
-        <v>-8.1</v>
+        <v>-1.4</v>
       </c>
       <c r="F42" t="n">
-        <v>71.72</v>
+        <v>70.09</v>
       </c>
       <c r="G42" t="n">
-        <v>10.87</v>
+        <v>1.64</v>
       </c>
       <c r="H42" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>24-06-2026</t>
+          <t>29-05-2026</t>
         </is>
       </c>
     </row>
@@ -6947,7 +6947,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
@@ -6957,7 +6957,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10">
@@ -6967,7 +6967,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -6977,7 +6977,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>